<commit_message>
created bank bic lookup
</commit_message>
<xml_diff>
--- a/RTSIS-SUBMISSION-SEQUENCE-REPORT.xlsx
+++ b/RTSIS-SUBMISSION-SEQUENCE-REPORT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\mcb\rtsis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcb0168e\Desktop\mcb-rtsis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45918C28-9DDA-4117-B6C7-FEC672039052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1041410C-07B1-44D9-BE9B-7A30B354D9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Submission Sequence" sheetId="2" r:id="rId1"/>
@@ -1139,23 +1139,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M104"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
-    <col min="2" max="2" width="30.7109375" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" customWidth="1"/>
-    <col min="5" max="5" width="13.42578125" customWidth="1"/>
-    <col min="6" max="6" width="29.85546875" customWidth="1"/>
-    <col min="7" max="7" width="28.42578125" customWidth="1"/>
-    <col min="8" max="8" width="16.85546875" customWidth="1"/>
-    <col min="9" max="9" width="21.140625" customWidth="1"/>
-    <col min="10" max="10" width="27.5703125" customWidth="1"/>
-    <col min="11" max="11" width="20.140625" customWidth="1"/>
-    <col min="12" max="12" width="21.85546875" customWidth="1"/>
-    <col min="13" max="13" width="18.28515625" customWidth="1"/>
+    <col min="2" max="2" width="30.6640625" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="13.44140625" customWidth="1"/>
+    <col min="6" max="6" width="29.88671875" customWidth="1"/>
+    <col min="7" max="7" width="28.44140625" customWidth="1"/>
+    <col min="8" max="8" width="16.88671875" customWidth="1"/>
+    <col min="9" max="9" width="21.109375" customWidth="1"/>
+    <col min="10" max="10" width="27.5546875" customWidth="1"/>
+    <col min="11" max="11" width="20.109375" customWidth="1"/>
+    <col min="12" max="12" width="21.88671875" customWidth="1"/>
+    <col min="13" max="13" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="13.5">
+    <row r="1" spans="1:13" ht="13.8">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1196,7 +1196,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="13.5">
+    <row r="2" spans="1:13" ht="13.8">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1231,7 +1231,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="13.5">
+    <row r="3" spans="1:13" ht="13.8">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1266,7 +1266,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="13.5">
+    <row r="4" spans="1:13" ht="13.8">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1301,7 +1301,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="13.5">
+    <row r="5" spans="1:13" ht="13.8">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1336,7 +1336,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="13.5">
+    <row r="6" spans="1:13" ht="13.8">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1371,7 +1371,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="13.5">
+    <row r="7" spans="1:13" ht="13.8">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1406,7 +1406,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="13.5">
+    <row r="8" spans="1:13" ht="13.8">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="13.5">
+    <row r="9" spans="1:13" ht="13.8">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="13.5">
+    <row r="10" spans="1:13" ht="13.8">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1481,7 +1481,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="13.5">
+    <row r="11" spans="1:13" ht="13.8">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="13.5">
+    <row r="12" spans="1:13" ht="13.8">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1523,7 +1523,7 @@
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
     </row>
-    <row r="13" spans="1:13" ht="13.5">
+    <row r="13" spans="1:13" ht="13.8">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1543,7 +1543,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="13.5">
+    <row r="14" spans="1:13" ht="13.8">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1563,7 +1563,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="13.5">
+    <row r="15" spans="1:13" ht="13.8">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1598,7 +1598,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="13.5">
+    <row r="16" spans="1:13" ht="13.8">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1618,7 +1618,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="13.5">
+    <row r="17" spans="1:13" ht="13.8">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="13.5">
+    <row r="18" spans="1:13" ht="13.8">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1688,7 +1688,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="13.5">
+    <row r="19" spans="1:13" ht="13.8">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1723,7 +1723,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="13.5">
+    <row r="20" spans="1:13" ht="13.8">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1758,7 +1758,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="13.5">
+    <row r="21" spans="1:13" ht="13.8">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1793,7 +1793,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="13.5">
+    <row r="22" spans="1:13" ht="13.8">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1828,7 +1828,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="13.5">
+    <row r="23" spans="1:13" ht="13.8">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1863,7 +1863,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="13.5">
+    <row r="24" spans="1:13" ht="13.8">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1898,7 +1898,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="13.5">
+    <row r="25" spans="1:13" ht="13.8">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1933,7 +1933,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="26" spans="1:13" s="15" customFormat="1" ht="15">
+    <row r="26" spans="1:13" s="15" customFormat="1" ht="14.4">
       <c r="A26" s="14">
         <v>25</v>
       </c>
@@ -1968,7 +1968,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="13.5">
+    <row r="27" spans="1:13" ht="13.8">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1988,7 +1988,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="13.5">
+    <row r="28" spans="1:13" ht="13.8">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -2008,7 +2008,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="13.5">
+    <row r="29" spans="1:13" ht="13.8">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -2028,7 +2028,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="13.5">
+    <row r="30" spans="1:13" ht="13.8">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -2048,7 +2048,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="13.5">
+    <row r="31" spans="1:13" ht="13.8">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="13.5">
+    <row r="32" spans="1:13" ht="13.8">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -2088,7 +2088,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="13.5">
+    <row r="33" spans="1:13" ht="13.8">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -2108,7 +2108,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="13.5">
+    <row r="34" spans="1:13" ht="13.8">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -2128,7 +2128,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="35" spans="1:13" ht="13.5">
+    <row r="35" spans="1:13" ht="13.8">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -2148,7 +2148,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="36" spans="1:13" ht="13.5">
+    <row r="36" spans="1:13" ht="13.8">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2168,7 +2168,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="13.5">
+    <row r="37" spans="1:13" ht="13.8">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -2188,7 +2188,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="13.5">
+    <row r="38" spans="1:13" ht="13.8">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -2208,7 +2208,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="13.5">
+    <row r="39" spans="1:13" ht="13.8">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -2243,7 +2243,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="13.5">
+    <row r="40" spans="1:13" ht="13.8">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -2278,7 +2278,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="41" spans="1:13" s="15" customFormat="1" ht="15">
+    <row r="41" spans="1:13" s="15" customFormat="1" ht="14.4">
       <c r="A41" s="14">
         <v>40</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="13.5">
+    <row r="42" spans="1:13" ht="13.8">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="13.5">
+    <row r="43" spans="1:13" ht="13.8">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -2353,7 +2353,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="13.5">
+    <row r="44" spans="1:13" ht="13.8">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -2373,7 +2373,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="45" spans="1:13" ht="13.5">
+    <row r="45" spans="1:13" ht="13.8">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -2393,7 +2393,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="13.5">
+    <row r="46" spans="1:13" ht="13.8">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -2413,7 +2413,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="47" spans="1:13" ht="13.5">
+    <row r="47" spans="1:13" ht="13.8">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -2433,7 +2433,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="48" spans="1:13" ht="13.5">
+    <row r="48" spans="1:13" ht="13.8">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -2453,7 +2453,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="49" spans="1:13" ht="13.5">
+    <row r="49" spans="1:13" ht="13.8">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="50" spans="1:13" ht="13.5">
+    <row r="50" spans="1:13" ht="13.8">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -2508,7 +2508,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="51" spans="1:13" ht="13.5">
+    <row r="51" spans="1:13" ht="13.8">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -2543,7 +2543,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="52" spans="1:13" ht="13.5">
+    <row r="52" spans="1:13" ht="13.8">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -2563,7 +2563,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="53" spans="1:13" ht="13.5">
+    <row r="53" spans="1:13" ht="13.8">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -2583,7 +2583,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="13.5">
+    <row r="54" spans="1:13" ht="13.8">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -2603,7 +2603,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="55" spans="1:13" ht="13.5">
+    <row r="55" spans="1:13" ht="13.8">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -2623,7 +2623,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="56" spans="1:13" ht="13.5">
+    <row r="56" spans="1:13" ht="13.8">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -2643,7 +2643,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="57" spans="1:13" ht="13.5">
+    <row r="57" spans="1:13" ht="13.8">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -2663,7 +2663,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="58" spans="1:13" ht="27">
+    <row r="58" spans="1:13" ht="27.6">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -2683,7 +2683,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="13.5">
+    <row r="59" spans="1:13" ht="13.8">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -2703,7 +2703,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="60" spans="1:13" ht="13.5">
+    <row r="60" spans="1:13" ht="13.8">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -2723,7 +2723,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="61" spans="1:13" ht="13.5">
+    <row r="61" spans="1:13" ht="13.8">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -2743,7 +2743,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="62" spans="1:13" ht="13.5">
+    <row r="62" spans="1:13" ht="13.8">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -2763,7 +2763,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="63" spans="1:13" ht="13.5">
+    <row r="63" spans="1:13" ht="13.8">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -2783,7 +2783,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="64" spans="1:13" ht="13.5">
+    <row r="64" spans="1:13" ht="13.8">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -2803,7 +2803,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="65" spans="1:13" ht="13.5">
+    <row r="65" spans="1:13" ht="13.8">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -2823,7 +2823,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="66" spans="1:13" ht="13.5">
+    <row r="66" spans="1:13" ht="13.8">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -2843,7 +2843,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="67" spans="1:13" ht="13.5">
+    <row r="67" spans="1:13" ht="13.8">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="68" spans="1:13" ht="13.5">
+    <row r="68" spans="1:13" ht="13.8">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -2883,7 +2883,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="69" spans="1:13" ht="13.5">
+    <row r="69" spans="1:13" ht="13.8">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -2903,7 +2903,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="70" spans="1:13" ht="13.5">
+    <row r="70" spans="1:13" ht="13.8">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -2923,7 +2923,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="71" spans="1:13" ht="13.5">
+    <row r="71" spans="1:13" ht="13.8">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -2943,7 +2943,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" spans="1:13" ht="13.5">
+    <row r="72" spans="1:13" ht="13.8">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -2963,7 +2963,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" spans="1:13" ht="13.5">
+    <row r="73" spans="1:13" ht="13.8">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -2983,7 +2983,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="74" spans="1:13" ht="13.5">
+    <row r="74" spans="1:13" ht="13.8">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -3018,7 +3018,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="75" spans="1:13" ht="13.5">
+    <row r="75" spans="1:13" ht="13.8">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -3038,7 +3038,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="76" spans="1:13" ht="13.5">
+    <row r="76" spans="1:13" ht="13.8">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -3073,7 +3073,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="77" spans="1:13" s="16" customFormat="1" ht="15">
+    <row r="77" spans="1:13" s="16" customFormat="1" ht="14.4">
       <c r="A77" s="16">
         <v>76</v>
       </c>
@@ -3108,7 +3108,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="78" spans="1:13" ht="15">
+    <row r="78" spans="1:13" ht="14.4">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -3143,7 +3143,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="79" spans="1:13" ht="13.5">
+    <row r="79" spans="1:13" ht="13.8">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -3178,7 +3178,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="80" spans="1:13" ht="13.5">
+    <row r="80" spans="1:13" ht="13.8">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -3213,7 +3213,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="81" spans="1:13" ht="13.5">
+    <row r="81" spans="1:13" ht="13.8">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -3248,7 +3248,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="82" spans="1:13" s="15" customFormat="1" ht="15">
+    <row r="82" spans="1:13" s="15" customFormat="1" ht="14.4">
       <c r="A82" s="14">
         <v>81</v>
       </c>
@@ -3283,7 +3283,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="83" spans="1:13" s="15" customFormat="1" ht="15">
+    <row r="83" spans="1:13" s="15" customFormat="1" ht="14.4">
       <c r="A83" s="14">
         <v>82</v>
       </c>
@@ -3318,7 +3318,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="84" spans="1:13" s="15" customFormat="1" ht="15">
+    <row r="84" spans="1:13" s="15" customFormat="1" ht="14.4">
       <c r="A84" s="14">
         <v>83</v>
       </c>
@@ -3353,7 +3353,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="85" spans="1:13" ht="13.5">
+    <row r="85" spans="1:13" ht="13.8">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -3388,7 +3388,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="86" spans="1:13" ht="13.5">
+    <row r="86" spans="1:13" ht="13.8">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -3408,7 +3408,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="87" spans="1:13" ht="13.5">
+    <row r="87" spans="1:13" ht="13.8">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -3428,7 +3428,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="88" spans="1:13" ht="13.5">
+    <row r="88" spans="1:13" ht="13.8">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -3448,7 +3448,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="89" spans="1:13" ht="13.5">
+    <row r="89" spans="1:13" ht="13.8">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -3468,7 +3468,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="90" spans="1:13" ht="13.5">
+    <row r="90" spans="1:13" ht="13.8">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -3503,7 +3503,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="91" spans="1:13" ht="13.5">
+    <row r="91" spans="1:13" ht="13.8">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -3523,7 +3523,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="92" spans="1:13" ht="13.5">
+    <row r="92" spans="1:13" ht="13.8">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -3558,7 +3558,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="93" spans="1:13" ht="13.5">
+    <row r="93" spans="1:13" ht="13.8">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -3593,7 +3593,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="94" spans="1:13" ht="13.5">
+    <row r="94" spans="1:13" ht="13.8">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -3613,7 +3613,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="95" spans="1:13" ht="13.5">
+    <row r="95" spans="1:13" ht="13.8">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -3633,7 +3633,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="96" spans="1:13" ht="13.5">
+    <row r="96" spans="1:13" ht="13.8">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -3653,7 +3653,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="97" spans="1:12" s="15" customFormat="1" ht="15">
+    <row r="97" spans="1:12" s="15" customFormat="1" ht="14.4">
       <c r="A97" s="14">
         <v>96</v>
       </c>
@@ -3688,7 +3688,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="100" spans="1:12" ht="15">
+    <row r="100" spans="1:12" ht="14.4">
       <c r="G100" s="19"/>
       <c r="H100" s="19" t="s">
         <v>176</v>
@@ -3697,7 +3697,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="101" spans="1:12" ht="15">
+    <row r="101" spans="1:12" ht="14.4">
       <c r="G101" s="19" t="s">
         <v>178</v>
       </c>
@@ -3708,7 +3708,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="102" spans="1:12" ht="15">
+    <row r="102" spans="1:12" ht="14.4">
       <c r="G102" s="19" t="s">
         <v>179</v>
       </c>
@@ -3719,7 +3719,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="103" spans="1:12" ht="15">
+    <row r="103" spans="1:12" ht="14.4">
       <c r="G103" s="19" t="s">
         <v>41</v>
       </c>
@@ -3730,7 +3730,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="104" spans="1:12" ht="15">
+    <row r="104" spans="1:12" ht="14.4">
       <c r="G104" s="19"/>
       <c r="H104" s="19"/>
       <c r="I104" s="19"/>

</xml_diff>

<commit_message>
added new more folders on pipeline
</commit_message>
<xml_diff>
--- a/RTSIS-SUBMISSION-SEQUENCE-REPORT.xlsx
+++ b/RTSIS-SUBMISSION-SEQUENCE-REPORT.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcb0168e\Desktop\mcb-rtsis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1041410C-07B1-44D9-BE9B-7A30B354D9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500556E3-D788-4897-B01F-7578AE9236A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="180">
   <si>
     <t>S/No</t>
   </si>
@@ -595,7 +595,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -695,6 +695,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF00B050"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -760,7 +766,7 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -800,6 +806,7 @@
     <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="4" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Bad" xfId="3" builtinId="27"/>
@@ -2187,6 +2194,9 @@
       <c r="F37" t="s">
         <v>129</v>
       </c>
+      <c r="J37" s="21" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="38" spans="1:13" ht="13.8">
       <c r="A38" s="2">

</xml_diff>

<commit_message>
introduction to channel report
</commit_message>
<xml_diff>
--- a/RTSIS-SUBMISSION-SEQUENCE-REPORT.xlsx
+++ b/RTSIS-SUBMISSION-SEQUENCE-REPORT.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mcb0168e\Desktop\mcb-rtsis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\mcb\rtsis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500556E3-D788-4897-B01F-7578AE9236A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C39158FF-5A74-463C-B90E-7735A558E7A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Submission Sequence" sheetId="2" r:id="rId1"/>
@@ -702,7 +702,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -723,6 +723,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -766,7 +772,7 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -807,6 +813,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Bad" xfId="3" builtinId="27"/>
@@ -1146,23 +1162,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M104"/>
-  <sheetFormatPr defaultRowHeight="13.2"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="2" max="2" width="30.6640625" customWidth="1"/>
-    <col min="3" max="3" width="17.44140625" customWidth="1"/>
-    <col min="4" max="4" width="12.33203125" customWidth="1"/>
-    <col min="5" max="5" width="13.44140625" customWidth="1"/>
-    <col min="6" max="6" width="29.88671875" customWidth="1"/>
-    <col min="7" max="7" width="28.44140625" customWidth="1"/>
-    <col min="8" max="8" width="16.88671875" customWidth="1"/>
-    <col min="9" max="9" width="21.109375" customWidth="1"/>
-    <col min="10" max="10" width="27.5546875" customWidth="1"/>
-    <col min="11" max="11" width="20.109375" customWidth="1"/>
-    <col min="12" max="12" width="21.88671875" customWidth="1"/>
-    <col min="13" max="13" width="18.33203125" customWidth="1"/>
+    <col min="2" max="2" width="30.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.42578125" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" customWidth="1"/>
+    <col min="5" max="5" width="13.42578125" customWidth="1"/>
+    <col min="6" max="6" width="29.85546875" customWidth="1"/>
+    <col min="7" max="7" width="28.42578125" customWidth="1"/>
+    <col min="8" max="8" width="16.85546875" customWidth="1"/>
+    <col min="9" max="9" width="21.140625" customWidth="1"/>
+    <col min="10" max="10" width="27.5703125" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" customWidth="1"/>
+    <col min="12" max="12" width="21.85546875" customWidth="1"/>
+    <col min="13" max="13" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="13.8">
+    <row r="1" spans="1:13" ht="13.5">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1203,7 +1219,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="13.8">
+    <row r="2" spans="1:13" ht="13.5">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1238,7 +1254,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="13.8">
+    <row r="3" spans="1:13" ht="13.5">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1273,7 +1289,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="13.8">
+    <row r="4" spans="1:13" ht="13.5">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1308,7 +1324,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="13.8">
+    <row r="5" spans="1:13" ht="13.5">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1343,7 +1359,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="13.8">
+    <row r="6" spans="1:13" ht="13.5">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1378,7 +1394,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="13.8">
+    <row r="7" spans="1:13" ht="13.5">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1413,7 +1429,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="13.8">
+    <row r="8" spans="1:13" ht="13.5">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1433,7 +1449,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="13.8">
+    <row r="9" spans="1:13" ht="13.5">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1453,7 +1469,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="13.8">
+    <row r="10" spans="1:13" ht="13.5">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1488,7 +1504,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="13.8">
+    <row r="11" spans="1:13" ht="13.5">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1508,7 +1524,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="13.8">
+    <row r="12" spans="1:13" ht="13.5">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1530,7 +1546,7 @@
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
     </row>
-    <row r="13" spans="1:13" ht="13.8">
+    <row r="13" spans="1:13" ht="13.5">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1550,7 +1566,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="13.8">
+    <row r="14" spans="1:13" ht="13.5">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1570,7 +1586,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="13.8">
+    <row r="15" spans="1:13" ht="13.5">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1605,7 +1621,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="13.8">
+    <row r="16" spans="1:13" ht="13.5">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1625,7 +1641,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="13.8">
+    <row r="17" spans="1:13" ht="13.5">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1660,7 +1676,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="13.8">
+    <row r="18" spans="1:13" ht="13.5">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1695,7 +1711,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="13.8">
+    <row r="19" spans="1:13" ht="13.5">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1730,7 +1746,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="13.8">
+    <row r="20" spans="1:13" ht="13.5">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1765,7 +1781,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="13.8">
+    <row r="21" spans="1:13" ht="13.5">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1800,7 +1816,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="13.8">
+    <row r="22" spans="1:13" ht="13.5">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1835,7 +1851,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="13.8">
+    <row r="23" spans="1:13" ht="13.5">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1870,7 +1886,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="13.8">
+    <row r="24" spans="1:13" ht="13.5">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1905,7 +1921,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="13.8">
+    <row r="25" spans="1:13" ht="13.5">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1940,7 +1956,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="26" spans="1:13" s="15" customFormat="1" ht="14.4">
+    <row r="26" spans="1:13" s="15" customFormat="1" ht="15">
       <c r="A26" s="14">
         <v>25</v>
       </c>
@@ -1975,7 +1991,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="13.8">
+    <row r="27" spans="1:13" ht="13.5">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1995,7 +2011,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="13.8">
+    <row r="28" spans="1:13" ht="13.5">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -2015,7 +2031,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="13.8">
+    <row r="29" spans="1:13" ht="13.5">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -2035,7 +2051,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="13.8">
+    <row r="30" spans="1:13" ht="13.5">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -2055,7 +2071,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="13.8">
+    <row r="31" spans="1:13" ht="13.5">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -2075,7 +2091,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="13.8">
+    <row r="32" spans="1:13" ht="13.5">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -2095,7 +2111,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="13.8">
+    <row r="33" spans="1:13" ht="13.5">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -2115,7 +2131,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="13.8">
+    <row r="34" spans="1:13" ht="13.5">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -2135,7 +2151,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="35" spans="1:13" ht="13.8">
+    <row r="35" spans="1:13" ht="13.5">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -2155,7 +2171,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="36" spans="1:13" ht="13.8">
+    <row r="36" spans="1:13" ht="13.5">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2175,7 +2191,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="13.8">
+    <row r="37" spans="1:13" ht="13.5">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -2198,7 +2214,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="13.8">
+    <row r="38" spans="1:13" ht="13.5">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -2218,7 +2234,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="13.8">
+    <row r="39" spans="1:13" ht="13.5">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -2253,42 +2269,42 @@
         <v>170</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="13.8">
-      <c r="A40" s="2">
+    <row r="40" spans="1:13" s="25" customFormat="1" ht="13.5">
+      <c r="A40" s="22">
         <v>39</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" s="23" t="s">
         <v>45</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="D40" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E40" s="4">
+      <c r="D40" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="E40" s="24">
         <v>10</v>
       </c>
-      <c r="F40" t="s">
+      <c r="F40" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="G40" s="7" t="s">
+      <c r="G40" s="26" t="s">
         <v>154</v>
       </c>
-      <c r="H40" s="7" t="s">
+      <c r="H40" s="26" t="s">
         <v>155</v>
       </c>
-      <c r="I40" t="s">
+      <c r="I40" s="25" t="s">
         <v>159</v>
       </c>
-      <c r="J40" s="13" t="s">
+      <c r="J40" s="27" t="s">
         <v>167</v>
       </c>
-      <c r="M40" t="s">
+      <c r="M40" s="25" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="41" spans="1:13" s="15" customFormat="1" ht="14.4">
+    <row r="41" spans="1:13" s="15" customFormat="1" ht="15">
       <c r="A41" s="14">
         <v>40</v>
       </c>
@@ -2323,7 +2339,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="13.8">
+    <row r="42" spans="1:13" ht="13.5">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2343,7 +2359,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="13.8">
+    <row r="43" spans="1:13" ht="13.5">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -2363,7 +2379,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="13.8">
+    <row r="44" spans="1:13" ht="13.5">
       <c r="A44" s="2">
         <v>43</v>
       </c>
@@ -2383,7 +2399,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="45" spans="1:13" ht="13.8">
+    <row r="45" spans="1:13" ht="13.5">
       <c r="A45" s="2">
         <v>44</v>
       </c>
@@ -2403,7 +2419,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="13.8">
+    <row r="46" spans="1:13" ht="13.5">
       <c r="A46" s="2">
         <v>45</v>
       </c>
@@ -2423,7 +2439,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="47" spans="1:13" ht="13.8">
+    <row r="47" spans="1:13" ht="13.5">
       <c r="A47" s="2">
         <v>46</v>
       </c>
@@ -2443,7 +2459,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="48" spans="1:13" ht="13.8">
+    <row r="48" spans="1:13" ht="13.5">
       <c r="A48" s="2">
         <v>47</v>
       </c>
@@ -2463,7 +2479,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="49" spans="1:13" ht="13.8">
+    <row r="49" spans="1:13" ht="13.5">
       <c r="A49" s="2">
         <v>48</v>
       </c>
@@ -2498,7 +2514,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="50" spans="1:13" ht="13.8">
+    <row r="50" spans="1:13" ht="13.5">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -2518,7 +2534,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="51" spans="1:13" ht="13.8">
+    <row r="51" spans="1:13" ht="13.5">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -2553,7 +2569,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="52" spans="1:13" ht="13.8">
+    <row r="52" spans="1:13" ht="13.5">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -2573,7 +2589,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="53" spans="1:13" ht="13.8">
+    <row r="53" spans="1:13" ht="13.5">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -2593,7 +2609,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="13.8">
+    <row r="54" spans="1:13" ht="13.5">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -2613,7 +2629,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="55" spans="1:13" ht="13.8">
+    <row r="55" spans="1:13" ht="13.5">
       <c r="A55" s="2">
         <v>54</v>
       </c>
@@ -2633,7 +2649,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="56" spans="1:13" ht="13.8">
+    <row r="56" spans="1:13" ht="13.5">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -2653,7 +2669,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="57" spans="1:13" ht="13.8">
+    <row r="57" spans="1:13" ht="13.5">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -2673,7 +2689,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="58" spans="1:13" ht="27.6">
+    <row r="58" spans="1:13" ht="27">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -2693,7 +2709,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="13.8">
+    <row r="59" spans="1:13" ht="13.5">
       <c r="A59" s="2">
         <v>58</v>
       </c>
@@ -2713,7 +2729,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="60" spans="1:13" ht="13.8">
+    <row r="60" spans="1:13" ht="13.5">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -2733,7 +2749,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="61" spans="1:13" ht="13.8">
+    <row r="61" spans="1:13" ht="13.5">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -2753,7 +2769,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="62" spans="1:13" ht="13.8">
+    <row r="62" spans="1:13" ht="13.5">
       <c r="A62" s="2">
         <v>61</v>
       </c>
@@ -2773,7 +2789,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="63" spans="1:13" ht="13.8">
+    <row r="63" spans="1:13" ht="13.5">
       <c r="A63" s="2">
         <v>62</v>
       </c>
@@ -2793,7 +2809,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="64" spans="1:13" ht="13.8">
+    <row r="64" spans="1:13" ht="13.5">
       <c r="A64" s="2">
         <v>63</v>
       </c>
@@ -2813,7 +2829,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="65" spans="1:13" ht="13.8">
+    <row r="65" spans="1:13" ht="13.5">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -2833,7 +2849,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="66" spans="1:13" ht="13.8">
+    <row r="66" spans="1:13" ht="13.5">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -2853,7 +2869,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="67" spans="1:13" ht="13.8">
+    <row r="67" spans="1:13" ht="13.5">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -2873,7 +2889,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="68" spans="1:13" ht="13.8">
+    <row r="68" spans="1:13" ht="13.5">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -2893,7 +2909,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="69" spans="1:13" ht="13.8">
+    <row r="69" spans="1:13" ht="13.5">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -2913,7 +2929,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="70" spans="1:13" ht="13.8">
+    <row r="70" spans="1:13" ht="13.5">
       <c r="A70" s="2">
         <v>69</v>
       </c>
@@ -2933,7 +2949,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="71" spans="1:13" ht="13.8">
+    <row r="71" spans="1:13" ht="13.5">
       <c r="A71" s="2">
         <v>70</v>
       </c>
@@ -2953,7 +2969,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" spans="1:13" ht="13.8">
+    <row r="72" spans="1:13" ht="13.5">
       <c r="A72" s="2">
         <v>71</v>
       </c>
@@ -2973,7 +2989,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" spans="1:13" ht="13.8">
+    <row r="73" spans="1:13" ht="13.5">
       <c r="A73" s="2">
         <v>72</v>
       </c>
@@ -2993,7 +3009,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="74" spans="1:13" ht="13.8">
+    <row r="74" spans="1:13" ht="13.5">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -3028,7 +3044,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="75" spans="1:13" ht="13.8">
+    <row r="75" spans="1:13" ht="13.5">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -3048,7 +3064,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="76" spans="1:13" ht="13.8">
+    <row r="76" spans="1:13" ht="13.5">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -3083,7 +3099,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="77" spans="1:13" s="16" customFormat="1" ht="14.4">
+    <row r="77" spans="1:13" s="16" customFormat="1" ht="15">
       <c r="A77" s="16">
         <v>76</v>
       </c>
@@ -3118,7 +3134,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="78" spans="1:13" ht="14.4">
+    <row r="78" spans="1:13" ht="15">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -3153,7 +3169,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="79" spans="1:13" ht="13.8">
+    <row r="79" spans="1:13" ht="13.5">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -3188,7 +3204,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="80" spans="1:13" ht="13.8">
+    <row r="80" spans="1:13" ht="13.5">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -3223,7 +3239,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="81" spans="1:13" ht="13.8">
+    <row r="81" spans="1:13" ht="13.5">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -3258,7 +3274,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="82" spans="1:13" s="15" customFormat="1" ht="14.4">
+    <row r="82" spans="1:13" s="15" customFormat="1" ht="15">
       <c r="A82" s="14">
         <v>81</v>
       </c>
@@ -3293,7 +3309,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="83" spans="1:13" s="15" customFormat="1" ht="14.4">
+    <row r="83" spans="1:13" s="15" customFormat="1" ht="15">
       <c r="A83" s="14">
         <v>82</v>
       </c>
@@ -3328,7 +3344,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="84" spans="1:13" s="15" customFormat="1" ht="14.4">
+    <row r="84" spans="1:13" s="15" customFormat="1" ht="15">
       <c r="A84" s="14">
         <v>83</v>
       </c>
@@ -3363,7 +3379,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="85" spans="1:13" ht="13.8">
+    <row r="85" spans="1:13" ht="13.5">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -3398,7 +3414,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="86" spans="1:13" ht="13.8">
+    <row r="86" spans="1:13" ht="13.5">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -3418,7 +3434,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="87" spans="1:13" ht="13.8">
+    <row r="87" spans="1:13" ht="13.5">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -3438,7 +3454,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="88" spans="1:13" ht="13.8">
+    <row r="88" spans="1:13" ht="13.5">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -3458,7 +3474,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="89" spans="1:13" ht="13.8">
+    <row r="89" spans="1:13" ht="13.5">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -3478,7 +3494,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="90" spans="1:13" ht="13.8">
+    <row r="90" spans="1:13" ht="13.5">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -3513,7 +3529,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="91" spans="1:13" ht="13.8">
+    <row r="91" spans="1:13" ht="13.5">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -3533,7 +3549,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="92" spans="1:13" ht="13.8">
+    <row r="92" spans="1:13" ht="13.5">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -3568,7 +3584,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="93" spans="1:13" ht="13.8">
+    <row r="93" spans="1:13" ht="13.5">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -3603,7 +3619,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="94" spans="1:13" ht="13.8">
+    <row r="94" spans="1:13" ht="13.5">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -3623,7 +3639,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="95" spans="1:13" ht="13.8">
+    <row r="95" spans="1:13" ht="13.5">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -3643,7 +3659,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="96" spans="1:13" ht="13.8">
+    <row r="96" spans="1:13" ht="13.5">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -3663,7 +3679,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="97" spans="1:12" s="15" customFormat="1" ht="14.4">
+    <row r="97" spans="1:12" s="15" customFormat="1" ht="15">
       <c r="A97" s="14">
         <v>96</v>
       </c>
@@ -3698,7 +3714,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="100" spans="1:12" ht="14.4">
+    <row r="100" spans="1:12" ht="15">
       <c r="G100" s="19"/>
       <c r="H100" s="19" t="s">
         <v>176</v>
@@ -3707,7 +3723,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="101" spans="1:12" ht="14.4">
+    <row r="101" spans="1:12" ht="15">
       <c r="G101" s="19" t="s">
         <v>178</v>
       </c>
@@ -3718,7 +3734,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="102" spans="1:12" ht="14.4">
+    <row r="102" spans="1:12" ht="15">
       <c r="G102" s="19" t="s">
         <v>179</v>
       </c>
@@ -3729,7 +3745,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="103" spans="1:12" ht="14.4">
+    <row r="103" spans="1:12" ht="15">
       <c r="G103" s="19" t="s">
         <v>41</v>
       </c>
@@ -3740,7 +3756,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="104" spans="1:12" ht="14.4">
+    <row r="104" spans="1:12" ht="15">
       <c r="G104" s="19"/>
       <c r="H104" s="19"/>
       <c r="I104" s="19"/>

</xml_diff>